<commit_message>
Análisis clusters y case-mix inclussion
</commit_message>
<xml_diff>
--- a/Output/Tables/Access_model.xlsx
+++ b/Output/Tables/Access_model.xlsx
@@ -1,98 +1,94 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usr\Desktop\ATDOM_GIT\proyecto_atdom\Output\Tables\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41875B52-918D-4BCA-854B-9402388F0C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
-  <si>
-    <t>Home_based_PHC_org</t>
-  </si>
-  <si>
-    <t>M0: Crude</t>
-  </si>
-  <si>
-    <t>M1: Age + sex</t>
-  </si>
-  <si>
-    <t>M2: Age + sex + SES</t>
-  </si>
-  <si>
-    <t>Adjusted rate per 1,000</t>
-  </si>
-  <si>
-    <t>UAB consulta</t>
-  </si>
-  <si>
-    <t>1.00 (Ref.)</t>
-  </si>
-  <si>
-    <t>14.4 (12.7–16.3)</t>
-  </si>
-  <si>
-    <t>Equip ATDOM</t>
-  </si>
-  <si>
-    <t>1.13 (0.82–1.56)</t>
-  </si>
-  <si>
-    <t>1.47 (1.27–1.70)</t>
-  </si>
-  <si>
-    <t>1.45 (1.25–1.69)</t>
-  </si>
-  <si>
-    <t>20.9 (18.8–23.3)</t>
-  </si>
-  <si>
-    <t>Equip Inf</t>
-  </si>
-  <si>
-    <t>1.10 (0.72–1.67)</t>
-  </si>
-  <si>
-    <t>1.29 (1.08–1.54)</t>
-  </si>
-  <si>
-    <t>18.5 (16.2–21.2)</t>
-  </si>
-  <si>
-    <t>UAB consulta reforç</t>
-  </si>
-  <si>
-    <t>1.04 (0.76–1.42)</t>
-  </si>
-  <si>
-    <t>1.45 (1.27–1.67)</t>
-  </si>
-  <si>
-    <t>1.48 (1.28–1.72)</t>
-  </si>
-  <si>
-    <t>21.4 (19.3–23.7)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t xml:space="preserve">Home_based_PHC_org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M0: Crude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1: Age + sex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M2: Age + sex + SES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjusted rate per 1,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAB consulta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.00 (Ref.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14.4 (12.7–16.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equip ATDOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.13 (0.82–1.56)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.47 (1.27–1.70)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.45 (1.25–1.69)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.9 (18.7–23.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equip Inf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.10 (0.73–1.67)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.30 (1.09–1.55)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.29 (1.08–1.54)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.5 (16.2–21.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAB consulta reforç</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.04 (0.77–1.42)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.46 (1.27–1.68)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.49 (1.28–1.72)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.4 (19.3–23.7)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -128,15 +124,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -418,15 +405,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="5" width="23.140625" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -443,7 +426,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -460,7 +443,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -477,7 +460,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -488,31 +471,31 @@
         <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>